<commit_message>
feat(models,eval,calibration): market eval CLV separation, canonical beta calibration, MLB v9 v4, WNBA & Tennis derivative pricing
</commit_message>
<xml_diff>
--- a/data/archive/2026-08-30-ncaaf-synthetic-main-quarantine/flat_ncaaf.xlsx
+++ b/data/archive/2026-08-30-ncaaf-synthetic-main-quarantine/flat_ncaaf.xlsx
@@ -1817,13 +1817,13 @@
         </is>
       </c>
       <c r="L2" s="26" t="n">
-        <v>100</v>
+        <v>-125</v>
       </c>
       <c r="M2" s="27" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="N2" s="28" t="n">
-        <v>0.5</v>
+        <v>0.555556</v>
       </c>
       <c r="O2" s="28" t="n">
         <v>0.550101</v>
@@ -1866,7 +1866,7 @@
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
       <c r="AC2" s="30" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
         <is>
@@ -2131,13 +2131,13 @@
         </is>
       </c>
       <c r="L3" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M3" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N3" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O3" s="28" t="n">
         <v>0.834067</v>
@@ -2180,7 +2180,7 @@
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
       <c r="AC3" s="30" t="n">
-        <v>2</v>
+        <v>1.8182</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
         <is>
@@ -2447,13 +2447,13 @@
         </is>
       </c>
       <c r="L4" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M4" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N4" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O4" s="28" t="n">
         <v>0.875533</v>
@@ -3365,13 +3365,13 @@
         </is>
       </c>
       <c r="L7" s="26" t="n">
-        <v>100</v>
+        <v>-900</v>
       </c>
       <c r="M7" s="27" t="n">
-        <v>2</v>
+        <v>1.111111</v>
       </c>
       <c r="N7" s="28" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="O7" s="28" t="n">
         <v>0.980205</v>
@@ -3414,7 +3414,7 @@
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
       <c r="AC7" s="30" t="n">
-        <v>2</v>
+        <v>0.2222</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         </is>
       </c>
       <c r="L8" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M8" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N8" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O8" s="28" t="n">
         <v>0.9828</v>
@@ -3728,7 +3728,7 @@
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
       <c r="AC8" s="30" t="n">
-        <v>2</v>
+        <v>1.8182</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
         <is>
@@ -3995,13 +3995,13 @@
         </is>
       </c>
       <c r="L9" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M9" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N9" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O9" s="28" t="n">
         <v>0.584467</v>
@@ -4309,13 +4309,13 @@
         </is>
       </c>
       <c r="L10" s="26" t="n">
-        <v>100</v>
+        <v>-125</v>
       </c>
       <c r="M10" s="27" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="N10" s="28" t="n">
-        <v>0.5</v>
+        <v>0.555556</v>
       </c>
       <c r="O10" s="28" t="n">
         <v>0.621685</v>
@@ -4358,7 +4358,7 @@
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
       <c r="AC10" s="30" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
         <is>
@@ -4623,13 +4623,13 @@
         </is>
       </c>
       <c r="L11" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M11" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N11" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O11" s="28" t="n">
         <v>0.5324</v>
@@ -4939,13 +4939,13 @@
         </is>
       </c>
       <c r="L12" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M12" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N12" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O12" s="28" t="n">
         <v>0.749867</v>
@@ -5253,13 +5253,13 @@
         </is>
       </c>
       <c r="L13" s="26" t="n">
-        <v>100</v>
+        <v>-250</v>
       </c>
       <c r="M13" s="27" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="N13" s="28" t="n">
-        <v>0.5</v>
+        <v>0.714286</v>
       </c>
       <c r="O13" s="28" t="n">
         <v>0.774213</v>
@@ -5567,13 +5567,13 @@
         </is>
       </c>
       <c r="L14" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M14" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N14" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O14" s="28" t="n">
         <v>0.9276</v>
@@ -5883,13 +5883,13 @@
         </is>
       </c>
       <c r="L15" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M15" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N15" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O15" s="28" t="n">
         <v>0.882333</v>
@@ -6197,13 +6197,13 @@
         </is>
       </c>
       <c r="L16" s="26" t="n">
-        <v>100</v>
+        <v>-250</v>
       </c>
       <c r="M16" s="27" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="N16" s="28" t="n">
-        <v>0.5</v>
+        <v>0.714286</v>
       </c>
       <c r="O16" s="28" t="n">
         <v>0.724011</v>
@@ -6246,7 +6246,7 @@
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
       <c r="AC16" s="30" t="n">
-        <v>1.25</v>
+        <v>0.5</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
         <is>
@@ -6511,13 +6511,13 @@
         </is>
       </c>
       <c r="L17" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M17" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N17" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O17" s="28" t="n">
         <v>0.6311330000000001</v>
@@ -6827,13 +6827,13 @@
         </is>
       </c>
       <c r="L18" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M18" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N18" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O18" s="28" t="n">
         <v>0.724867</v>
@@ -7141,13 +7141,13 @@
         </is>
       </c>
       <c r="L19" s="26" t="n">
-        <v>100</v>
+        <v>-900</v>
       </c>
       <c r="M19" s="27" t="n">
-        <v>2</v>
+        <v>1.111111</v>
       </c>
       <c r="N19" s="28" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="O19" s="28" t="n">
         <v>0.911523</v>
@@ -7190,7 +7190,7 @@
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
       <c r="AC19" s="30" t="n">
-        <v>2</v>
+        <v>0.2222</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
         <is>
@@ -7455,13 +7455,13 @@
         </is>
       </c>
       <c r="L20" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M20" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N20" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O20" s="28" t="n">
         <v>0.8070000000000001</v>
@@ -7504,7 +7504,7 @@
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n"/>
       <c r="AC20" s="30" t="n">
-        <v>1.75</v>
+        <v>1.5909</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
         <is>
@@ -7771,13 +7771,13 @@
         </is>
       </c>
       <c r="L21" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M21" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N21" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O21" s="28" t="n">
         <v>0.858067</v>
@@ -7820,7 +7820,7 @@
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
       <c r="AC21" s="30" t="n">
-        <v>2</v>
+        <v>1.8182</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
         <is>
@@ -8085,13 +8085,13 @@
         </is>
       </c>
       <c r="L22" s="26" t="n">
-        <v>100</v>
+        <v>-900</v>
       </c>
       <c r="M22" s="27" t="n">
-        <v>2</v>
+        <v>1.111111</v>
       </c>
       <c r="N22" s="28" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="O22" s="28" t="n">
         <v>0.938717</v>
@@ -8134,7 +8134,7 @@
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n"/>
       <c r="AC22" s="30" t="n">
-        <v>2</v>
+        <v>0.2222</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
         <is>
@@ -8399,13 +8399,13 @@
         </is>
       </c>
       <c r="L23" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M23" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N23" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O23" s="28" t="n">
         <v>0.974267</v>
@@ -8448,7 +8448,7 @@
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
       <c r="AC23" s="30" t="n">
-        <v>2</v>
+        <v>1.8182</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
         <is>
@@ -8715,13 +8715,13 @@
         </is>
       </c>
       <c r="L24" s="26" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="M24" s="27" t="n">
-        <v>2</v>
+        <v>1.909091</v>
       </c>
       <c r="N24" s="28" t="n">
-        <v>0.5</v>
+        <v>0.52381</v>
       </c>
       <c r="O24" s="28" t="n">
         <v>0.6126</v>

</xml_diff>